<commit_message>
fix: BROKERAGE_AUTH_ID typo, code 1011 fallback, remove extra quote fetch
</commit_message>
<xml_diff>
--- a/PaperTrade_Journal.xlsx
+++ b/PaperTrade_Journal.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,16 +489,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-08 08:31:40</t>
+          <t>2026-05-15 14:59:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GME</t>
+          <t>BNZI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -507,17 +512,17 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>24.04</v>
+        <v>8.01</v>
       </c>
       <c r="F2" t="n">
-        <v>24.3076</v>
+        <v>8.0313</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.2676</v>
+        <v>0.0213</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -533,284 +538,9 @@
           <t>OPEN</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-08 08:32:34</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MARA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>13</v>
-      </c>
-      <c r="E3" t="n">
-        <v>12.69</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12.8183</v>
-      </c>
-      <c r="G3" t="n">
-        <v>12.3662</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.1283</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.1238</v>
-      </c>
-      <c r="J3" t="n">
-        <v>-5.8773</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Volume Spike (&gt;300%)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-08 09:07:40</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>34.04</v>
-      </c>
-      <c r="F4" t="n">
-        <v>34.2258</v>
-      </c>
-      <c r="G4" t="n">
-        <v>34.2899</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1858</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1201</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.3205</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Volume Spike (&gt;300%)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-08 09:31:07</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>34.48</v>
-      </c>
-      <c r="F5" t="n">
-        <v>34.9694</v>
-      </c>
-      <c r="G5" t="n">
-        <v>35.0375</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.4894</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.3405</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Volume Spike (&gt;300%)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-08 10:13:28</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NFLX</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>87.79000000000001</v>
-      </c>
-      <c r="F6" t="n">
-        <v>88.27120000000001</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>0.4812</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Volume Spike (&gt;300%)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-05-08 11:43:35</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>MARA</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>15</v>
-      </c>
-      <c r="E7" t="n">
-        <v>12.83</v>
-      </c>
-      <c r="F7" t="n">
-        <v>12.8854</v>
-      </c>
-      <c r="G7" t="n">
-        <v>12.8736</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0554</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.0564</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-0.177</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>EMA Crossover (9 &gt; 21)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-05-08 14:56:29</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>RIOT</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" t="n">
-        <v>24.06</v>
-      </c>
-      <c r="F8" t="n">
-        <v>24.3389</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>0.2789</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Volume Spike (&gt;300%)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
         </is>
       </c>
     </row>

</xml_diff>